<commit_message>
18.03.2026: updated mapping file
</commit_message>
<xml_diff>
--- a/mapping.xlsx
+++ b/mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub Repos\DEPI-Final-Project---Gold-and-Oil-Predictions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA35CF39-BA2B-48EC-A635-F349363A5B17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1844E932-810E-4CB1-BB68-79193D0A6AEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{64DC8462-31C8-413C-AE04-A946F8DA8A48}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{64DC8462-31C8-413C-AE04-A946F8DA8A48}"/>
   </bookViews>
   <sheets>
     <sheet name="Cleaned Tables Mapping" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="43">
   <si>
     <t>No.</t>
   </si>
@@ -156,6 +156,15 @@
   </si>
   <si>
     <t>china_shanghai_prices</t>
+  </si>
+  <si>
+    <t>global_gpr_index</t>
+  </si>
+  <si>
+    <t>global_ai_gpr_index</t>
+  </si>
+  <si>
+    <t>matteoiacoviello</t>
   </si>
 </sst>
 </file>
@@ -553,12 +562,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93370650-F311-4D2E-A663-3DC42763697A}">
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="48.28515625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1016,6 +1025,38 @@
       </c>
       <c r="E30" s="1"/>
     </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
+        <f>SUBTOTAL(3,$C$4:C31)</f>
+        <v>28</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E31" s="1"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <f>SUBTOTAL(3,$C$4:C32)</f>
+        <v>29</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E32" s="1"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
18/03/2026: 1- added related macroeconomic data to euro zone. 2- updated mapping file to reflect point (1) changes.
</commit_message>
<xml_diff>
--- a/mapping.xlsx
+++ b/mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub Repos\DEPI-Final-Project---Gold-and-Oil-Predictions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1844E932-810E-4CB1-BB68-79193D0A6AEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{086A0318-F764-4B13-98D7-31BA0DFADEF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{64DC8462-31C8-413C-AE04-A946F8DA8A48}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="47">
   <si>
     <t>No.</t>
   </si>
@@ -165,6 +165,18 @@
   </si>
   <si>
     <t>matteoiacoviello</t>
+  </si>
+  <si>
+    <t>euro_gdp_rate</t>
+  </si>
+  <si>
+    <t>euro_inflation_rate</t>
+  </si>
+  <si>
+    <t>euro_interest_rate</t>
+  </si>
+  <si>
+    <t>ECB</t>
   </si>
 </sst>
 </file>
@@ -562,7 +574,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93370650-F311-4D2E-A663-3DC42763697A}">
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20.5703125" bestFit="1" customWidth="1"/>
@@ -1057,6 +1069,54 @@
       </c>
       <c r="E32" s="1"/>
     </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="1">
+        <f>SUBTOTAL(3,$C$4:C33)</f>
+        <v>30</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E33" s="1"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
+        <f>SUBTOTAL(3,$C$4:C34)</f>
+        <v>31</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E34" s="1"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
+        <f>SUBTOTAL(3,$C$4:C35)</f>
+        <v>32</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E35" s="1"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>